<commit_message>
feat: update category and product templates for improved styling and readability; refactor URL paths for consistency
</commit_message>
<xml_diff>
--- a/bulk_up/plantilla_categories.xlsx
+++ b/bulk_up/plantilla_categories.xlsx
@@ -1,21 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Robert\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Apudig\Proyecto\apudig_mvp\bulk_up\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B6C6BAD-F442-423D-B6B4-BEDE2D18B923}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62EEDECF-7AAA-46CB-AF16-65663370DD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41730" yWindow="1245" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="plantilla" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -406,10 +411,10 @@
     <t>INODOROS, URINARIOS Y LAVATORIOS</t>
   </si>
   <si>
-    <t>1401</t>
-  </si>
-  <si>
     <t>PEGAMENTOS PARA PISO Y ACCESORIOS</t>
+  </si>
+  <si>
+    <t>PC01</t>
   </si>
 </sst>
 </file>
@@ -1500,10 +1505,10 @@
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="B64" s="11" t="s">
         <v>128</v>
-      </c>
-      <c r="B64" s="11" t="s">
-        <v>129</v>
       </c>
       <c r="C64" s="10" t="s">
         <v>3</v>

</xml_diff>